<commit_message>
Add eval suite and tests; fix habit ranking and sample calibration
- Eval harness: fixed cases, seeded sweeps per habit, clean-control
  false-positive check, copy/consistency checks and a ship bar, plus a
  held-out seed set (SEED_OFFSET=2000) not used for tuning.
- Unit tests for symbols, timestamps, round-trip rebuild and the
  example workbook.
- Engine: prefer a narrower nested habit (expiry-day inside an
  instrument), re-check significance on residual trades, stricter bar
  for multi-variant checks, measure holding-losers against quick losses
  not explained by other habits, re-rank by final cost.
- Sample tradebook regenerated with the fair holding-losers definition.
- UI: drop duplicate open-position / skipped-row notes.
</commit_message>
<xml_diff>
--- a/app/public/samples/sept-2026-tradebook.xlsx
+++ b/app/public/samples/sept-2026-tradebook.xlsx
@@ -510,7 +510,7 @@
         <v>30</v>
       </c>
       <c r="J3">
-        <v>216.1</v>
+        <v>216.3</v>
       </c>
       <c r="K3" t="str">
         <v>10482021</v>
@@ -551,7 +551,7 @@
         <v>30</v>
       </c>
       <c r="J4">
-        <v>216.5</v>
+        <v>216.7</v>
       </c>
       <c r="K4" t="str">
         <v>10482044</v>
@@ -592,7 +592,7 @@
         <v>30</v>
       </c>
       <c r="J5">
-        <v>216.5</v>
+        <v>216.7</v>
       </c>
       <c r="K5" t="str">
         <v>10482082</v>
@@ -1166,7 +1166,7 @@
         <v>150</v>
       </c>
       <c r="J19">
-        <v>1502.05</v>
+        <v>1501.95</v>
       </c>
       <c r="K19" t="str">
         <v>10482475</v>
@@ -1371,7 +1371,7 @@
         <v>150</v>
       </c>
       <c r="J24">
-        <v>1524.9</v>
+        <v>1525.05</v>
       </c>
       <c r="K24" t="str">
         <v>10482589</v>
@@ -1535,7 +1535,7 @@
         <v>200</v>
       </c>
       <c r="J28">
-        <v>993.8</v>
+        <v>990.5</v>
       </c>
       <c r="K28" t="str">
         <v>10482637</v>
@@ -1699,7 +1699,7 @@
         <v>200</v>
       </c>
       <c r="J32">
-        <v>999.45</v>
+        <v>999.75</v>
       </c>
       <c r="K32" t="str">
         <v>10482742</v>
@@ -1945,7 +1945,7 @@
         <v>150</v>
       </c>
       <c r="J38">
-        <v>1525.6</v>
+        <v>1525.75</v>
       </c>
       <c r="K38" t="str">
         <v>10482874</v>
@@ -2109,7 +2109,7 @@
         <v>100</v>
       </c>
       <c r="J42">
-        <v>1005.35</v>
+        <v>1005.55</v>
       </c>
       <c r="K42" t="str">
         <v>10483000</v>
@@ -2150,7 +2150,7 @@
         <v>100</v>
       </c>
       <c r="J43">
-        <v>1005.35</v>
+        <v>1005.55</v>
       </c>
       <c r="K43" t="str">
         <v>10483037</v>
@@ -2232,7 +2232,7 @@
         <v>130</v>
       </c>
       <c r="J45">
-        <v>138.65</v>
+        <v>138.8</v>
       </c>
       <c r="K45" t="str">
         <v>10483083</v>
@@ -2273,7 +2273,7 @@
         <v>65</v>
       </c>
       <c r="J46">
-        <v>139.55</v>
+        <v>139.7</v>
       </c>
       <c r="K46" t="str">
         <v>10483093</v>
@@ -2355,7 +2355,7 @@
         <v>200</v>
       </c>
       <c r="J48">
-        <v>1004.6</v>
+        <v>1004.9</v>
       </c>
       <c r="K48" t="str">
         <v>10483155</v>
@@ -2560,7 +2560,7 @@
         <v>150</v>
       </c>
       <c r="J53">
-        <v>1489</v>
+        <v>1489.15</v>
       </c>
       <c r="K53" t="str">
         <v>10483295</v>
@@ -2642,7 +2642,7 @@
         <v>150</v>
       </c>
       <c r="J55">
-        <v>1481.65</v>
+        <v>1481.55</v>
       </c>
       <c r="K55" t="str">
         <v>10483313</v>
@@ -3011,7 +3011,7 @@
         <v>200</v>
       </c>
       <c r="J64">
-        <v>995.8</v>
+        <v>996</v>
       </c>
       <c r="K64" t="str">
         <v>10483518</v>
@@ -3257,7 +3257,7 @@
         <v>90</v>
       </c>
       <c r="J70">
-        <v>308.6</v>
+        <v>308.95</v>
       </c>
       <c r="K70" t="str">
         <v>10483631</v>
@@ -3421,7 +3421,7 @@
         <v>150</v>
       </c>
       <c r="J74">
-        <v>1503.5</v>
+        <v>1503.7</v>
       </c>
       <c r="K74" t="str">
         <v>10483736</v>
@@ -3585,7 +3585,7 @@
         <v>70</v>
       </c>
       <c r="J78">
-        <v>1007.1</v>
+        <v>1007.3</v>
       </c>
       <c r="K78" t="str">
         <v>10483825</v>
@@ -3626,7 +3626,7 @@
         <v>70</v>
       </c>
       <c r="J79">
-        <v>1007.25</v>
+        <v>1007.45</v>
       </c>
       <c r="K79" t="str">
         <v>10483840</v>
@@ -3667,7 +3667,7 @@
         <v>60</v>
       </c>
       <c r="J80">
-        <v>1007.25</v>
+        <v>1007.45</v>
       </c>
       <c r="K80" t="str">
         <v>10483877</v>
@@ -3749,7 +3749,7 @@
         <v>90</v>
       </c>
       <c r="J82">
-        <v>380.15</v>
+        <v>380.35</v>
       </c>
       <c r="K82" t="str">
         <v>10483940</v>
@@ -4200,7 +4200,7 @@
         <v>90</v>
       </c>
       <c r="J93">
-        <v>183.1</v>
+        <v>183.35</v>
       </c>
       <c r="K93" t="str">
         <v>10484166</v>
@@ -4364,7 +4364,7 @@
         <v>195</v>
       </c>
       <c r="J97">
-        <v>82.1</v>
+        <v>82.25</v>
       </c>
       <c r="K97" t="str">
         <v>10484249</v>
@@ -4446,7 +4446,7 @@
         <v>90</v>
       </c>
       <c r="J99">
-        <v>232.4</v>
+        <v>232.6</v>
       </c>
       <c r="K99" t="str">
         <v>10484290</v>
@@ -5143,7 +5143,7 @@
         <v>200</v>
       </c>
       <c r="J116">
-        <v>998.7</v>
+        <v>998.9</v>
       </c>
       <c r="K116" t="str">
         <v>10484715</v>
@@ -5307,7 +5307,7 @@
         <v>195</v>
       </c>
       <c r="J120">
-        <v>104.9</v>
+        <v>105.2</v>
       </c>
       <c r="K120" t="str">
         <v>10484796</v>
@@ -5389,7 +5389,7 @@
         <v>90</v>
       </c>
       <c r="J122">
-        <v>347</v>
+        <v>347.3</v>
       </c>
       <c r="K122" t="str">
         <v>10484825</v>
@@ -5553,7 +5553,7 @@
         <v>130</v>
       </c>
       <c r="J126">
-        <v>248.2</v>
+        <v>248.45</v>
       </c>
       <c r="K126" t="str">
         <v>10484911</v>
@@ -5594,7 +5594,7 @@
         <v>65</v>
       </c>
       <c r="J127">
-        <v>248.8</v>
+        <v>249.05</v>
       </c>
       <c r="K127" t="str">
         <v>10484937</v>
@@ -5676,7 +5676,7 @@
         <v>150</v>
       </c>
       <c r="J129">
-        <v>1486.6</v>
+        <v>1486.75</v>
       </c>
       <c r="K129" t="str">
         <v>10484987</v>
@@ -5799,7 +5799,7 @@
         <v>150</v>
       </c>
       <c r="J132">
-        <v>1489.6</v>
+        <v>1489.7</v>
       </c>
       <c r="K132" t="str">
         <v>10485084</v>
@@ -5881,7 +5881,7 @@
         <v>195</v>
       </c>
       <c r="J134">
-        <v>235.15</v>
+        <v>235.4</v>
       </c>
       <c r="K134" t="str">
         <v>10485113</v>
@@ -6004,7 +6004,7 @@
         <v>90</v>
       </c>
       <c r="J137">
-        <v>408.45</v>
+        <v>408.6</v>
       </c>
       <c r="K137" t="str">
         <v>10485152</v>
@@ -6373,7 +6373,7 @@
         <v>200</v>
       </c>
       <c r="J146">
-        <v>1000.2</v>
+        <v>1000.4</v>
       </c>
       <c r="K146" t="str">
         <v>10485380</v>
@@ -6455,7 +6455,7 @@
         <v>195</v>
       </c>
       <c r="J148">
-        <v>107.45</v>
+        <v>107.75</v>
       </c>
       <c r="K148" t="str">
         <v>10485401</v>
@@ -6701,7 +6701,7 @@
         <v>130</v>
       </c>
       <c r="J154">
-        <v>97.15</v>
+        <v>97.4</v>
       </c>
       <c r="K154" t="str">
         <v>10485556</v>
@@ -6742,7 +6742,7 @@
         <v>65</v>
       </c>
       <c r="J155">
-        <v>97.2</v>
+        <v>97.45</v>
       </c>
       <c r="K155" t="str">
         <v>10485594</v>
@@ -6824,7 +6824,7 @@
         <v>90</v>
       </c>
       <c r="J157">
-        <v>343</v>
+        <v>343.25</v>
       </c>
       <c r="K157" t="str">
         <v>10485658</v>
@@ -6906,7 +6906,7 @@
         <v>90</v>
       </c>
       <c r="J159">
-        <v>176.7</v>
+        <v>176.95</v>
       </c>
       <c r="K159" t="str">
         <v>10485678</v>
@@ -7357,7 +7357,7 @@
         <v>90</v>
       </c>
       <c r="J170">
-        <v>366.75</v>
+        <v>367</v>
       </c>
       <c r="K170" t="str">
         <v>10485937</v>
@@ -7767,7 +7767,7 @@
         <v>130</v>
       </c>
       <c r="J180">
-        <v>144.2</v>
+        <v>144.3</v>
       </c>
       <c r="K180" t="str">
         <v>10486083</v>
@@ -7808,7 +7808,7 @@
         <v>65</v>
       </c>
       <c r="J181">
-        <v>144.5</v>
+        <v>144.6</v>
       </c>
       <c r="K181" t="str">
         <v>10486097</v>
@@ -7972,7 +7972,7 @@
         <v>150</v>
       </c>
       <c r="J185">
-        <v>1470.9</v>
+        <v>1470.85</v>
       </c>
       <c r="K185" t="str">
         <v>10486176</v>
@@ -8218,7 +8218,7 @@
         <v>90</v>
       </c>
       <c r="J191">
-        <v>293.55</v>
+        <v>293.8</v>
       </c>
       <c r="K191" t="str">
         <v>10486307</v>
@@ -8382,7 +8382,7 @@
         <v>60</v>
       </c>
       <c r="J195">
-        <v>188.7</v>
+        <v>188.9</v>
       </c>
       <c r="K195" t="str">
         <v>10486398</v>
@@ -8423,7 +8423,7 @@
         <v>30</v>
       </c>
       <c r="J196">
-        <v>189.15</v>
+        <v>189.35</v>
       </c>
       <c r="K196" t="str">
         <v>10486420</v>
@@ -8546,7 +8546,7 @@
         <v>195</v>
       </c>
       <c r="J199">
-        <v>118.7</v>
+        <v>118.85</v>
       </c>
       <c r="K199" t="str">
         <v>10486474</v>
@@ -8669,7 +8669,7 @@
         <v>60</v>
       </c>
       <c r="J202">
-        <v>412.9</v>
+        <v>413.05</v>
       </c>
       <c r="K202" t="str">
         <v>10486544</v>
@@ -8710,7 +8710,7 @@
         <v>30</v>
       </c>
       <c r="J203">
-        <v>413.35</v>
+        <v>413.5</v>
       </c>
       <c r="K203" t="str">
         <v>10486565</v>
@@ -8792,7 +8792,7 @@
         <v>195</v>
       </c>
       <c r="J205">
-        <v>208.7</v>
+        <v>208.9</v>
       </c>
       <c r="K205" t="str">
         <v>10486596</v>
@@ -8874,7 +8874,7 @@
         <v>130</v>
       </c>
       <c r="J207">
-        <v>209.1</v>
+        <v>209.3</v>
       </c>
       <c r="K207" t="str">
         <v>10486629</v>
@@ -8915,7 +8915,7 @@
         <v>65</v>
       </c>
       <c r="J208">
-        <v>209.15</v>
+        <v>209.35</v>
       </c>
       <c r="K208" t="str">
         <v>10486632</v>
@@ -9202,7 +9202,7 @@
         <v>200</v>
       </c>
       <c r="J215">
-        <v>1003.55</v>
+        <v>1003.8</v>
       </c>
       <c r="K215" t="str">
         <v>10486770</v>
@@ -9325,7 +9325,7 @@
         <v>90</v>
       </c>
       <c r="J218">
-        <v>195.95</v>
+        <v>196.1</v>
       </c>
       <c r="K218" t="str">
         <v>10486856</v>
@@ -9448,7 +9448,7 @@
         <v>90</v>
       </c>
       <c r="J221">
-        <v>302.2</v>
+        <v>302.4</v>
       </c>
       <c r="K221" t="str">
         <v>10486936</v>
@@ -9735,7 +9735,7 @@
         <v>65</v>
       </c>
       <c r="J228">
-        <v>192</v>
+        <v>192.25</v>
       </c>
       <c r="K228" t="str">
         <v>10487091</v>
@@ -9776,7 +9776,7 @@
         <v>65</v>
       </c>
       <c r="J229">
-        <v>191.85</v>
+        <v>192.1</v>
       </c>
       <c r="K229" t="str">
         <v>10487106</v>
@@ -9817,7 +9817,7 @@
         <v>65</v>
       </c>
       <c r="J230">
-        <v>192</v>
+        <v>192.25</v>
       </c>
       <c r="K230" t="str">
         <v>10487127</v>
@@ -9981,7 +9981,7 @@
         <v>90</v>
       </c>
       <c r="J234">
-        <v>307.05</v>
+        <v>307.35</v>
       </c>
       <c r="K234" t="str">
         <v>10487177</v>
@@ -10145,7 +10145,7 @@
         <v>130</v>
       </c>
       <c r="J238">
-        <v>66.3</v>
+        <v>66.4</v>
       </c>
       <c r="K238" t="str">
         <v>10487305</v>
@@ -10186,7 +10186,7 @@
         <v>65</v>
       </c>
       <c r="J239">
-        <v>66.3</v>
+        <v>66.4</v>
       </c>
       <c r="K239" t="str">
         <v>10487342</v>
@@ -10473,7 +10473,7 @@
         <v>195</v>
       </c>
       <c r="J246">
-        <v>200.7</v>
+        <v>201.05</v>
       </c>
       <c r="K246" t="str">
         <v>10487503</v>
@@ -10637,7 +10637,7 @@
         <v>150</v>
       </c>
       <c r="J250">
-        <v>1489.5</v>
+        <v>1488</v>
       </c>
       <c r="K250" t="str">
         <v>10487605</v>
@@ -10678,7 +10678,7 @@
         <v>130</v>
       </c>
       <c r="J251">
-        <v>120</v>
+        <v>120.25</v>
       </c>
       <c r="K251" t="str">
         <v>10487634</v>
@@ -10719,7 +10719,7 @@
         <v>65</v>
       </c>
       <c r="J252">
-        <v>120</v>
+        <v>120.25</v>
       </c>
       <c r="K252" t="str">
         <v>10487653</v>
@@ -10801,7 +10801,7 @@
         <v>200</v>
       </c>
       <c r="J254">
-        <v>1009.85</v>
+        <v>1010.05</v>
       </c>
       <c r="K254" t="str">
         <v>10487706</v>
@@ -11211,7 +11211,7 @@
         <v>90</v>
       </c>
       <c r="J264">
-        <v>343.9</v>
+        <v>344.2</v>
       </c>
       <c r="K264" t="str">
         <v>10487894</v>
@@ -11703,7 +11703,7 @@
         <v>195</v>
       </c>
       <c r="J276">
-        <v>90.3</v>
+        <v>90.4</v>
       </c>
       <c r="K276" t="str">
         <v>10488093</v>
@@ -12113,7 +12113,7 @@
         <v>80</v>
       </c>
       <c r="J286">
-        <v>1512.05</v>
+        <v>1512.15</v>
       </c>
       <c r="K286" t="str">
         <v>10488346</v>
@@ -12154,7 +12154,7 @@
         <v>70</v>
       </c>
       <c r="J287">
-        <v>1512.05</v>
+        <v>1512.15</v>
       </c>
       <c r="K287" t="str">
         <v>10488363</v>
@@ -12277,7 +12277,7 @@
         <v>200</v>
       </c>
       <c r="J290">
-        <v>999.55</v>
+        <v>999.25</v>
       </c>
       <c r="K290" t="str">
         <v>10488418</v>
@@ -12318,7 +12318,7 @@
         <v>195</v>
       </c>
       <c r="J291">
-        <v>136.5</v>
+        <v>131.95</v>
       </c>
       <c r="K291" t="str">
         <v>10488442</v>
@@ -12523,7 +12523,7 @@
         <v>150</v>
       </c>
       <c r="J296">
-        <v>1508.95</v>
+        <v>1509.05</v>
       </c>
       <c r="K296" t="str">
         <v>10488528</v>
@@ -12687,7 +12687,7 @@
         <v>30</v>
       </c>
       <c r="J300">
-        <v>388.6</v>
+        <v>388.95</v>
       </c>
       <c r="K300" t="str">
         <v>10488614</v>
@@ -12728,7 +12728,7 @@
         <v>30</v>
       </c>
       <c r="J301">
-        <v>388.9</v>
+        <v>389.25</v>
       </c>
       <c r="K301" t="str">
         <v>10488648</v>
@@ -12769,7 +12769,7 @@
         <v>30</v>
       </c>
       <c r="J302">
-        <v>388.9</v>
+        <v>389.25</v>
       </c>
       <c r="K302" t="str">
         <v>10488666</v>
@@ -12933,7 +12933,7 @@
         <v>90</v>
       </c>
       <c r="J306">
-        <v>352.1</v>
+        <v>352.4</v>
       </c>
       <c r="K306" t="str">
         <v>10488771</v>
@@ -13261,7 +13261,7 @@
         <v>200</v>
       </c>
       <c r="J314">
-        <v>1013.6</v>
+        <v>1013.85</v>
       </c>
       <c r="K314" t="str">
         <v>10488917</v>
@@ -13343,7 +13343,7 @@
         <v>130</v>
       </c>
       <c r="J316">
-        <v>119.65</v>
+        <v>119.85</v>
       </c>
       <c r="K316" t="str">
         <v>10488977</v>
@@ -13384,7 +13384,7 @@
         <v>65</v>
       </c>
       <c r="J317">
-        <v>120.55</v>
+        <v>120.75</v>
       </c>
       <c r="K317" t="str">
         <v>10489004</v>
@@ -13507,7 +13507,7 @@
         <v>195</v>
       </c>
       <c r="J320">
-        <v>201.75</v>
+        <v>202</v>
       </c>
       <c r="K320" t="str">
         <v>10489077</v>
@@ -13589,7 +13589,7 @@
         <v>200</v>
       </c>
       <c r="J322">
-        <v>1010.75</v>
+        <v>1011.05</v>
       </c>
       <c r="K322" t="str">
         <v>10489126</v>
@@ -13958,7 +13958,7 @@
         <v>90</v>
       </c>
       <c r="J331">
-        <v>209.3</v>
+        <v>209.4</v>
       </c>
       <c r="K331" t="str">
         <v>10489263</v>
@@ -14040,7 +14040,7 @@
         <v>90</v>
       </c>
       <c r="J333">
-        <v>296.15</v>
+        <v>296.35</v>
       </c>
       <c r="K333" t="str">
         <v>10489323</v>
@@ -14122,7 +14122,7 @@
         <v>195</v>
       </c>
       <c r="J335">
-        <v>101.15</v>
+        <v>101.35</v>
       </c>
       <c r="K335" t="str">
         <v>10489377</v>
@@ -14204,7 +14204,7 @@
         <v>195</v>
       </c>
       <c r="J337">
-        <v>201.45</v>
+        <v>201.7</v>
       </c>
       <c r="K337" t="str">
         <v>10489437</v>
@@ -14491,7 +14491,7 @@
         <v>90</v>
       </c>
       <c r="J344">
-        <v>222</v>
+        <v>222.2</v>
       </c>
       <c r="K344" t="str">
         <v>10489591</v>
@@ -14696,7 +14696,7 @@
         <v>70</v>
       </c>
       <c r="J349">
-        <v>1008</v>
+        <v>1008.2</v>
       </c>
       <c r="K349" t="str">
         <v>10489655</v>
@@ -14737,7 +14737,7 @@
         <v>70</v>
       </c>
       <c r="J350">
-        <v>1007.75</v>
+        <v>1007.95</v>
       </c>
       <c r="K350" t="str">
         <v>10489658</v>
@@ -14778,7 +14778,7 @@
         <v>60</v>
       </c>
       <c r="J351">
-        <v>1008</v>
+        <v>1008.2</v>
       </c>
       <c r="K351" t="str">
         <v>10489673</v>
@@ -15393,7 +15393,7 @@
         <v>90</v>
       </c>
       <c r="J366">
-        <v>361.7</v>
+        <v>361.95</v>
       </c>
       <c r="K366" t="str">
         <v>10490007</v>
@@ -15557,7 +15557,7 @@
         <v>90</v>
       </c>
       <c r="J370">
-        <v>400.85</v>
+        <v>401</v>
       </c>
       <c r="K370" t="str">
         <v>10490101</v>
@@ -15639,7 +15639,7 @@
         <v>130</v>
       </c>
       <c r="J372">
-        <v>81.75</v>
+        <v>81.85</v>
       </c>
       <c r="K372" t="str">
         <v>10490125</v>
@@ -15680,7 +15680,7 @@
         <v>65</v>
       </c>
       <c r="J373">
-        <v>81.8</v>
+        <v>81.9</v>
       </c>
       <c r="K373" t="str">
         <v>10490143</v>
@@ -15885,7 +15885,7 @@
         <v>90</v>
       </c>
       <c r="J378">
-        <v>348.4</v>
+        <v>342.8</v>
       </c>
       <c r="K378" t="str">
         <v>10490280</v>
@@ -15967,7 +15967,7 @@
         <v>100</v>
       </c>
       <c r="J380">
-        <v>997.65</v>
+        <v>997.9</v>
       </c>
       <c r="K380" t="str">
         <v>10490292</v>
@@ -16008,7 +16008,7 @@
         <v>100</v>
       </c>
       <c r="J381">
-        <v>997.65</v>
+        <v>997.9</v>
       </c>
       <c r="K381" t="str">
         <v>10490306</v>
@@ -16172,7 +16172,7 @@
         <v>195</v>
       </c>
       <c r="J385">
-        <v>185.9</v>
+        <v>186.15</v>
       </c>
       <c r="K385" t="str">
         <v>10490409</v>

</xml_diff>